<commit_message>
Update sql_prompt: CTE WO lintas bulan, larangan in_tcare
</commit_message>
<xml_diff>
--- a/Output/Sawa/Rekap/rekap_sawa.xlsx
+++ b/Output/Sawa/Rekap/rekap_sawa.xlsx
@@ -41660,17 +41660,17 @@
       </c>
       <c r="N469" t="inlineStr">
         <is>
+          <t>NASMOCO - TEGAL</t>
+        </is>
+      </c>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>2024-12-12</t>
+        </is>
+      </c>
+      <c r="P469" t="inlineStr">
+        <is>
           <t>NASMOCO SILIWANGI</t>
-        </is>
-      </c>
-      <c r="O469" t="inlineStr">
-        <is>
-          <t>2024-12-12</t>
-        </is>
-      </c>
-      <c r="P469" t="inlineStr">
-        <is>
-          <t>NASMOCO - TEGAL</t>
         </is>
       </c>
       <c r="Q469" t="inlineStr">

</xml_diff>